<commit_message>
✨ Separa Recebimento de Pagamento e leva OBs para aba de Pagamentos
</commit_message>
<xml_diff>
--- a/conciliacao.xlsx
+++ b/conciliacao.xlsx
@@ -1380,7 +1380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="10" min="1" max="1"/>
@@ -1390,6 +1390,8 @@
     <col width="13" customWidth="1" style="10" min="5" max="5"/>
     <col width="18" customWidth="1" style="10" min="6" max="6"/>
     <col width="32" customWidth="1" style="10" min="7" max="7"/>
+    <col width="14" customWidth="1" style="10" min="9" max="9"/>
+    <col width="14" customWidth="1" style="10" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1428,6 +1430,16 @@
           <t>Justificativas - Não reconciliadas</t>
         </is>
       </c>
+      <c r="I1" s="19" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="J1" s="19" t="inlineStr">
+        <is>
+          <t>VALOR</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="20" t="n">
@@ -1455,6 +1467,14 @@
         </is>
       </c>
       <c r="G2" s="21" t="n"/>
+      <c r="I2" s="20" t="inlineStr">
+        <is>
+          <t>183697</t>
+        </is>
+      </c>
+      <c r="J2" s="22" t="n">
+        <v>23771.75</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="n">
@@ -1482,6 +1502,14 @@
         </is>
       </c>
       <c r="G3" s="21" t="n"/>
+      <c r="I3" s="20" t="inlineStr">
+        <is>
+          <t>183698</t>
+        </is>
+      </c>
+      <c r="J3" s="22" t="n">
+        <v>364047.28</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="n">
@@ -1509,6 +1537,14 @@
         </is>
       </c>
       <c r="G4" s="21" t="n"/>
+      <c r="I4" s="20" t="inlineStr">
+        <is>
+          <t>183718</t>
+        </is>
+      </c>
+      <c r="J4" s="22" t="n">
+        <v>35472.8</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="n">
@@ -1536,6 +1572,14 @@
         </is>
       </c>
       <c r="G5" s="21" t="n"/>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>183720</t>
+        </is>
+      </c>
+      <c r="J5" s="22" t="n">
+        <v>19913.93</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n">
@@ -1563,6 +1607,14 @@
         </is>
       </c>
       <c r="G6" s="21" t="n"/>
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t>6825471</t>
+        </is>
+      </c>
+      <c r="J6" s="22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
@@ -1590,6 +1642,14 @@
         </is>
       </c>
       <c r="G7" s="21" t="n"/>
+      <c r="I7" s="20" t="inlineStr">
+        <is>
+          <t>6826209</t>
+        </is>
+      </c>
+      <c r="J7" s="22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="20" t="n">
@@ -1617,6 +1677,14 @@
         </is>
       </c>
       <c r="G8" s="21" t="n"/>
+      <c r="I8" s="20" t="inlineStr">
+        <is>
+          <t>6826210</t>
+        </is>
+      </c>
+      <c r="J8" s="22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n">
@@ -1644,6 +1712,14 @@
         </is>
       </c>
       <c r="G9" s="21" t="n"/>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="J9" s="22" t="n">
+        <v>545.78</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -1671,6 +1747,14 @@
         </is>
       </c>
       <c r="G10" s="21" t="n"/>
+      <c r="I10" s="20" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="J10" s="22" t="n">
+        <v>338.38</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n">
@@ -1698,6 +1782,14 @@
         </is>
       </c>
       <c r="G11" s="21" t="n"/>
+      <c r="I11" s="20" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="J11" s="22" t="n">
+        <v>184.21</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n">

</xml_diff>

<commit_message>
✨ OBs com VALOR=0 apagadas
</commit_message>
<xml_diff>
--- a/conciliacao.xlsx
+++ b/conciliacao.xlsx
@@ -96,7 +96,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -133,6 +133,7 @@
         <color rgb="00B7B7B7"/>
       </bottom>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -144,7 +145,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -212,6 +213,13 @@
     <xf numFmtId="4" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1609,11 +1617,11 @@
       <c r="G6" s="21" t="n"/>
       <c r="I6" s="20" t="inlineStr">
         <is>
-          <t>6825471</t>
+          <t>Pagamento</t>
         </is>
       </c>
       <c r="J6" s="22" t="n">
-        <v>0</v>
+        <v>545.78</v>
       </c>
     </row>
     <row r="7">
@@ -1644,11 +1652,11 @@
       <c r="G7" s="21" t="n"/>
       <c r="I7" s="20" t="inlineStr">
         <is>
-          <t>6826209</t>
+          <t>Pagamento</t>
         </is>
       </c>
       <c r="J7" s="22" t="n">
-        <v>0</v>
+        <v>338.38</v>
       </c>
     </row>
     <row r="8">
@@ -1679,11 +1687,11 @@
       <c r="G8" s="21" t="n"/>
       <c r="I8" s="20" t="inlineStr">
         <is>
-          <t>6826210</t>
+          <t>Pagamento</t>
         </is>
       </c>
       <c r="J8" s="22" t="n">
-        <v>0</v>
+        <v>184.21</v>
       </c>
     </row>
     <row r="9">
@@ -1712,14 +1720,8 @@
         </is>
       </c>
       <c r="G9" s="21" t="n"/>
-      <c r="I9" s="20" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="J9" s="22" t="n">
-        <v>545.78</v>
-      </c>
+      <c r="I9" s="23" t="n"/>
+      <c r="J9" s="24" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -1747,14 +1749,8 @@
         </is>
       </c>
       <c r="G10" s="21" t="n"/>
-      <c r="I10" s="20" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="J10" s="22" t="n">
-        <v>338.38</v>
-      </c>
+      <c r="I10" s="23" t="n"/>
+      <c r="J10" s="24" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n">
@@ -1782,14 +1778,8 @@
         </is>
       </c>
       <c r="G11" s="21" t="n"/>
-      <c r="I11" s="20" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="J11" s="22" t="n">
-        <v>184.21</v>
-      </c>
+      <c r="I11" s="23" t="n"/>
+      <c r="J11" s="24" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n">
@@ -1817,6 +1807,8 @@
         </is>
       </c>
       <c r="G12" s="21" t="n"/>
+      <c r="I12" s="25" t="n"/>
+      <c r="J12" s="25" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n">
@@ -1844,6 +1836,8 @@
         </is>
       </c>
       <c r="G13" s="21" t="n"/>
+      <c r="I13" s="25" t="n"/>
+      <c r="J13" s="25" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n">
@@ -1871,6 +1865,8 @@
         </is>
       </c>
       <c r="G14" s="21" t="n"/>
+      <c r="I14" s="25" t="n"/>
+      <c r="J14" s="25" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n">
@@ -1898,6 +1894,8 @@
         </is>
       </c>
       <c r="G15" s="21" t="n"/>
+      <c r="I15" s="25" t="n"/>
+      <c r="J15" s="25" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n">
@@ -1925,6 +1923,8 @@
         </is>
       </c>
       <c r="G16" s="21" t="n"/>
+      <c r="I16" s="25" t="n"/>
+      <c r="J16" s="25" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n">
@@ -1952,6 +1952,8 @@
         </is>
       </c>
       <c r="G17" s="21" t="n"/>
+      <c r="I17" s="25" t="n"/>
+      <c r="J17" s="25" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n">
@@ -1979,6 +1981,8 @@
         </is>
       </c>
       <c r="G18" s="21" t="n"/>
+      <c r="I18" s="25" t="n"/>
+      <c r="J18" s="25" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G18"/>

</xml_diff>

<commit_message>
✨ Relação entre Pagamentos e OBs funcionando
</commit_message>
<xml_diff>
--- a/conciliacao.xlsx
+++ b/conciliacao.xlsx
@@ -71,7 +71,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -93,6 +93,41 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CFE2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAD1DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D2E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE5CD"/>
       </patternFill>
     </fill>
   </fills>
@@ -145,7 +180,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -220,6 +255,69 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -712,7 +810,7 @@
         </is>
       </c>
       <c r="K5" s="17" t="n">
-        <v>19913.93</v>
+        <v>19919.93</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="10">
@@ -1388,7 +1486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="10" min="1" max="1"/>
@@ -1475,12 +1573,12 @@
         </is>
       </c>
       <c r="G2" s="21" t="n"/>
-      <c r="I2" s="20" t="inlineStr">
+      <c r="I2" s="26" t="inlineStr">
         <is>
           <t>183697</t>
         </is>
       </c>
-      <c r="J2" s="22" t="n">
+      <c r="J2" s="27" t="n">
         <v>23771.75</v>
       </c>
     </row>
@@ -1510,12 +1608,12 @@
         </is>
       </c>
       <c r="G3" s="21" t="n"/>
-      <c r="I3" s="20" t="inlineStr">
+      <c r="I3" s="28" t="inlineStr">
         <is>
           <t>183698</t>
         </is>
       </c>
-      <c r="J3" s="22" t="n">
+      <c r="J3" s="29" t="n">
         <v>364047.28</v>
       </c>
     </row>
@@ -1545,12 +1643,12 @@
         </is>
       </c>
       <c r="G4" s="21" t="n"/>
-      <c r="I4" s="20" t="inlineStr">
+      <c r="I4" s="30" t="inlineStr">
         <is>
           <t>183718</t>
         </is>
       </c>
-      <c r="J4" s="22" t="n">
+      <c r="J4" s="31" t="n">
         <v>35472.8</v>
       </c>
     </row>
@@ -1580,13 +1678,13 @@
         </is>
       </c>
       <c r="G5" s="21" t="n"/>
-      <c r="I5" s="20" t="inlineStr">
+      <c r="I5" s="32" t="inlineStr">
         <is>
           <t>183720</t>
         </is>
       </c>
-      <c r="J5" s="22" t="n">
-        <v>19913.93</v>
+      <c r="J5" s="33" t="n">
+        <v>19919.93</v>
       </c>
     </row>
     <row r="6">
@@ -1615,343 +1713,343 @@
         </is>
       </c>
       <c r="G6" s="21" t="n"/>
-      <c r="I6" s="20" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="J6" s="22" t="n">
+      <c r="I6" s="34" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="J6" s="35" t="n">
         <v>545.78</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="n">
+      <c r="A7" s="28" t="n">
         <v>10</v>
       </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="C7" s="21" t="n">
+      <c r="B7" s="36" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C7" s="36" t="n">
         <v>1040211</v>
       </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>27/jul/26</t>
-        </is>
-      </c>
-      <c r="E7" s="22" t="n">
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E7" s="29" t="n">
         <v>364047.28</v>
       </c>
-      <c r="F7" s="21" t="inlineStr">
-        <is>
-          <t>Não reconciliado</t>
-        </is>
-      </c>
-      <c r="G7" s="21" t="n"/>
-      <c r="I7" s="20" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="J7" s="22" t="n">
+      <c r="F7" s="36" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G7" s="36" t="n"/>
+      <c r="I7" s="37" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="J7" s="38" t="n">
         <v>338.38</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="n">
+      <c r="A8" s="30" t="n">
         <v>12</v>
       </c>
-      <c r="B8" s="21" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="C8" s="21" t="n">
+      <c r="B8" s="39" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C8" s="39" t="n">
         <v>1200393</v>
       </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t>27/jul/26</t>
-        </is>
-      </c>
-      <c r="E8" s="22" t="n">
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E8" s="31" t="n">
         <v>6236.25</v>
       </c>
-      <c r="F8" s="21" t="inlineStr">
-        <is>
-          <t>Não reconciliado</t>
-        </is>
-      </c>
-      <c r="G8" s="21" t="n"/>
-      <c r="I8" s="20" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="J8" s="22" t="n">
+      <c r="F8" s="39" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G8" s="39" t="n"/>
+      <c r="I8" s="40" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="J8" s="41" t="n">
         <v>184.21</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="n">
+      <c r="A9" s="30" t="n">
         <v>13</v>
       </c>
-      <c r="B9" s="21" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="C9" s="21" t="n">
+      <c r="B9" s="39" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C9" s="39" t="n">
         <v>1200393</v>
       </c>
-      <c r="D9" s="20" t="inlineStr">
-        <is>
-          <t>27/jul/26</t>
-        </is>
-      </c>
-      <c r="E9" s="22" t="n">
+      <c r="D9" s="30" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E9" s="31" t="n">
         <v>29236.55</v>
       </c>
-      <c r="F9" s="21" t="inlineStr">
-        <is>
-          <t>Não reconciliado</t>
-        </is>
-      </c>
-      <c r="G9" s="21" t="n"/>
+      <c r="F9" s="39" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G9" s="39" t="n"/>
       <c r="I9" s="23" t="n"/>
       <c r="J9" s="24" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="n">
+      <c r="A10" s="26" t="n">
         <v>14</v>
       </c>
-      <c r="B10" s="21" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="C10" s="21" t="n">
+      <c r="B10" s="42" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C10" s="42" t="n">
         <v>1200393</v>
       </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>27/jul/26</t>
-        </is>
-      </c>
-      <c r="E10" s="22" t="n">
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="n">
         <v>5853.45</v>
       </c>
-      <c r="F10" s="21" t="inlineStr">
-        <is>
-          <t>Não reconciliado</t>
-        </is>
-      </c>
-      <c r="G10" s="21" t="n"/>
+      <c r="F10" s="42" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G10" s="42" t="n"/>
       <c r="I10" s="23" t="n"/>
       <c r="J10" s="24" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="n">
+      <c r="A11" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="B11" s="21" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="C11" s="21" t="n">
+      <c r="B11" s="42" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C11" s="42" t="n">
         <v>1040211</v>
       </c>
-      <c r="D11" s="20" t="inlineStr">
-        <is>
-          <t>27/jul/26</t>
-        </is>
-      </c>
-      <c r="E11" s="22" t="n">
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E11" s="27" t="n">
         <v>17918.3</v>
       </c>
-      <c r="F11" s="21" t="inlineStr">
-        <is>
-          <t>Não reconciliado</t>
-        </is>
-      </c>
-      <c r="G11" s="21" t="n"/>
+      <c r="F11" s="42" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G11" s="42" t="n"/>
       <c r="I11" s="23" t="n"/>
       <c r="J11" s="24" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="n">
+      <c r="A12" s="37" t="n">
         <v>21</v>
       </c>
-      <c r="B12" s="21" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="C12" s="21" t="n">
+      <c r="B12" s="43" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C12" s="43" t="n">
         <v>1170144</v>
       </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>27/jul/26</t>
-        </is>
-      </c>
-      <c r="E12" s="22" t="n">
+      <c r="D12" s="37" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E12" s="38" t="n">
         <v>338.38</v>
       </c>
-      <c r="F12" s="21" t="inlineStr">
-        <is>
-          <t>Não reconciliado</t>
-        </is>
-      </c>
-      <c r="G12" s="21" t="n"/>
+      <c r="F12" s="43" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G12" s="43" t="n"/>
       <c r="I12" s="25" t="n"/>
       <c r="J12" s="25" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="n">
+      <c r="A13" s="32" t="n">
         <v>22</v>
       </c>
-      <c r="B13" s="21" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="C13" s="21" t="n">
+      <c r="B13" s="44" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C13" s="44" t="n">
         <v>1040109</v>
       </c>
-      <c r="D13" s="20" t="inlineStr">
-        <is>
-          <t>27/jul/26</t>
-        </is>
-      </c>
-      <c r="E13" s="22" t="n">
+      <c r="D13" s="32" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E13" s="33" t="n">
         <v>282.67</v>
       </c>
-      <c r="F13" s="21" t="inlineStr">
-        <is>
-          <t>Não reconciliado</t>
-        </is>
-      </c>
-      <c r="G13" s="21" t="n"/>
+      <c r="F13" s="44" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G13" s="44" t="n"/>
       <c r="I13" s="25" t="n"/>
       <c r="J13" s="25" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="n">
+      <c r="A14" s="32" t="n">
         <v>23</v>
       </c>
-      <c r="B14" s="21" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="C14" s="21" t="n">
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C14" s="44" t="n">
         <v>1040109</v>
       </c>
-      <c r="D14" s="20" t="inlineStr">
-        <is>
-          <t>27/jul/26</t>
-        </is>
-      </c>
-      <c r="E14" s="22" t="n">
+      <c r="D14" s="32" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E14" s="33" t="n">
         <v>19637.26</v>
       </c>
-      <c r="F14" s="21" t="inlineStr">
-        <is>
-          <t>Não reconciliado</t>
-        </is>
-      </c>
-      <c r="G14" s="21" t="n"/>
+      <c r="F14" s="44" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G14" s="44" t="n"/>
       <c r="I14" s="25" t="n"/>
       <c r="J14" s="25" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="n">
+      <c r="A15" s="40" t="n">
         <v>25</v>
       </c>
-      <c r="B15" s="21" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="C15" s="21" t="n">
+      <c r="B15" s="45" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C15" s="45" t="n">
         <v>1170144</v>
       </c>
-      <c r="D15" s="20" t="inlineStr">
-        <is>
-          <t>27/jul/26</t>
-        </is>
-      </c>
-      <c r="E15" s="22" t="n">
+      <c r="D15" s="40" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E15" s="41" t="n">
         <v>184.21</v>
       </c>
-      <c r="F15" s="21" t="inlineStr">
-        <is>
-          <t>Não reconciliado</t>
-        </is>
-      </c>
-      <c r="G15" s="21" t="n"/>
+      <c r="F15" s="45" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G15" s="45" t="n"/>
       <c r="I15" s="25" t="n"/>
       <c r="J15" s="25" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="n">
+      <c r="A16" s="34" t="n">
         <v>26</v>
       </c>
-      <c r="B16" s="21" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="C16" s="21" t="n">
+      <c r="B16" s="46" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C16" s="46" t="n">
         <v>1040375</v>
       </c>
-      <c r="D16" s="20" t="inlineStr">
-        <is>
-          <t>27/jul/26</t>
-        </is>
-      </c>
-      <c r="E16" s="22" t="n">
+      <c r="D16" s="34" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E16" s="35" t="n">
         <v>417.36</v>
       </c>
-      <c r="F16" s="21" t="inlineStr">
-        <is>
-          <t>Não reconciliado</t>
-        </is>
-      </c>
-      <c r="G16" s="21" t="n"/>
+      <c r="F16" s="46" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G16" s="46" t="n"/>
       <c r="I16" s="25" t="n"/>
       <c r="J16" s="25" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="n">
+      <c r="A17" s="34" t="n">
         <v>27</v>
       </c>
-      <c r="B17" s="21" t="inlineStr">
-        <is>
-          <t>Pagamento</t>
-        </is>
-      </c>
-      <c r="C17" s="21" t="n">
+      <c r="B17" s="46" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C17" s="46" t="n">
         <v>1040375</v>
       </c>
-      <c r="D17" s="20" t="inlineStr">
-        <is>
-          <t>27/jul/26</t>
-        </is>
-      </c>
-      <c r="E17" s="22" t="n">
+      <c r="D17" s="34" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E17" s="35" t="n">
         <v>128.42</v>
       </c>
-      <c r="F17" s="21" t="inlineStr">
-        <is>
-          <t>Não reconciliado</t>
-        </is>
-      </c>
-      <c r="G17" s="21" t="n"/>
+      <c r="F17" s="46" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G17" s="46" t="n"/>
       <c r="I17" s="25" t="n"/>
       <c r="J17" s="25" t="n"/>
     </row>
@@ -1984,6 +2082,7 @@
       <c r="I18" s="25" t="n"/>
       <c r="J18" s="25" t="n"/>
     </row>
+    <row r="19"/>
   </sheetData>
   <autoFilter ref="A1:G18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
✨ Separação de Recebimentos e Pagamentos na mesma aba
</commit_message>
<xml_diff>
--- a/conciliacao.xlsx
+++ b/conciliacao.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Conciliação" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Recebimentos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Pagamentos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Recebimentos e Pagamentos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Conciliação'!$A$1:$G$22</definedName>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -70,8 +71,14 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -130,8 +137,18 @@
         <fgColor rgb="00FCE5CD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E7D32"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B71C1C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -169,6 +186,20 @@
       </bottom>
     </border>
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="00B7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7B7B7"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -180,7 +211,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -318,6 +349,23 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1486,7 +1534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="10" min="1" max="1"/>
@@ -2082,9 +2130,801 @@
       <c r="I18" s="25" t="n"/>
       <c r="J18" s="25" t="n"/>
     </row>
-    <row r="19"/>
   </sheetData>
   <autoFilter ref="A1:G18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" style="10" min="1" max="1"/>
+    <col width="18" customWidth="1" style="10" min="2" max="2"/>
+    <col width="11" customWidth="1" style="10" min="3" max="3"/>
+    <col width="15" customWidth="1" style="10" min="4" max="4"/>
+    <col width="13" customWidth="1" style="10" min="5" max="5"/>
+    <col width="18" customWidth="1" style="10" min="6" max="6"/>
+    <col width="32" customWidth="1" style="10" min="7" max="7"/>
+    <col width="14" customWidth="1" style="10" min="9" max="9"/>
+    <col width="14" customWidth="1" style="10" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="47" t="inlineStr">
+        <is>
+          <t>RECEBIMENTOS (4)</t>
+        </is>
+      </c>
+      <c r="B1" s="48" t="n"/>
+      <c r="C1" s="48" t="n"/>
+      <c r="D1" s="48" t="n"/>
+      <c r="E1" s="48" t="n"/>
+      <c r="F1" s="48" t="n"/>
+      <c r="G1" s="48" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Linha</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C2" s="19" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="D2" s="19" t="inlineStr">
+        <is>
+          <t>Data Transação</t>
+        </is>
+      </c>
+      <c r="E2" s="19" t="inlineStr">
+        <is>
+          <t>Quantia</t>
+        </is>
+      </c>
+      <c r="F2" s="19" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G2" s="19" t="inlineStr">
+        <is>
+          <t>Justificativas - Não reconciliadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>Recebimento Div.</t>
+        </is>
+      </c>
+      <c r="C3" s="21" t="n">
+        <v>2130870</v>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E3" s="22" t="n">
+        <v>96587.98</v>
+      </c>
+      <c r="F3" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G3" s="21" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Recebimento</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="n">
+        <v>2090976</v>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E4" s="22" t="n">
+        <v>6979.7</v>
+      </c>
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G4" s="21" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>Recebimento Div.</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="n">
+        <v>2050900</v>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="n">
+        <v>184.21</v>
+      </c>
+      <c r="F5" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G5" s="21" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="49" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="50" t="inlineStr">
+        <is>
+          <t>Recebimento Div.</t>
+        </is>
+      </c>
+      <c r="C6" s="50" t="n">
+        <v>2140632</v>
+      </c>
+      <c r="D6" s="49" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E6" s="51" t="n">
+        <v>65543.33</v>
+      </c>
+      <c r="F6" s="50" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G6" s="50" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="52" t="inlineStr">
+        <is>
+          <t>PAGAMENTOS (17)</t>
+        </is>
+      </c>
+      <c r="B8" s="53" t="n"/>
+      <c r="C8" s="53" t="n"/>
+      <c r="D8" s="53" t="n"/>
+      <c r="E8" s="53" t="n"/>
+      <c r="F8" s="53" t="n"/>
+      <c r="G8" s="53" t="n"/>
+      <c r="I8" s="52" t="inlineStr">
+        <is>
+          <t>OB / VALOR</t>
+        </is>
+      </c>
+      <c r="J8" s="53" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Linha</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Data Transação</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>Quantia</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>Justificativas - Não reconciliadas</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>OB</t>
+        </is>
+      </c>
+      <c r="J9" s="19" t="inlineStr">
+        <is>
+          <t>VALOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento Div.</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="n">
+        <v>1040500</v>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E10" s="22" t="n">
+        <v>64.29000000000001</v>
+      </c>
+      <c r="F10" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G10" s="21" t="n"/>
+      <c r="I10" s="20" t="inlineStr">
+        <is>
+          <t>183697</t>
+        </is>
+      </c>
+      <c r="J10" s="22" t="n">
+        <v>23771.75</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento Div.</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="n">
+        <v>1040500</v>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E11" s="22" t="n">
+        <v>461.5</v>
+      </c>
+      <c r="F11" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G11" s="21" t="n"/>
+      <c r="I11" s="20" t="inlineStr">
+        <is>
+          <t>183698</t>
+        </is>
+      </c>
+      <c r="J11" s="22" t="n">
+        <v>364047.28</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento Div.</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="n">
+        <v>1040500</v>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E12" s="22" t="n">
+        <v>421.66</v>
+      </c>
+      <c r="F12" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G12" s="21" t="n"/>
+      <c r="I12" s="20" t="inlineStr">
+        <is>
+          <t>183718</t>
+        </is>
+      </c>
+      <c r="J12" s="22" t="n">
+        <v>35472.8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento Div.</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="n">
+        <v>1040500</v>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E13" s="22" t="n">
+        <v>586.76</v>
+      </c>
+      <c r="F13" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G13" s="21" t="n"/>
+      <c r="I13" s="20" t="inlineStr">
+        <is>
+          <t>183720</t>
+        </is>
+      </c>
+      <c r="J13" s="22" t="n">
+        <v>19919.93</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento Div.</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="n">
+        <v>1040500</v>
+      </c>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E14" s="22" t="n">
+        <v>488.04</v>
+      </c>
+      <c r="F14" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G14" s="21" t="n"/>
+      <c r="I14" s="20" t="inlineStr">
+        <is>
+          <t>6825471</t>
+        </is>
+      </c>
+      <c r="J14" s="22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="n">
+        <v>1040211</v>
+      </c>
+      <c r="D15" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E15" s="22" t="n">
+        <v>364047.28</v>
+      </c>
+      <c r="F15" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G15" s="21" t="n"/>
+      <c r="I15" s="20" t="inlineStr">
+        <is>
+          <t>6826209</t>
+        </is>
+      </c>
+      <c r="J15" s="22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="n">
+        <v>1200393</v>
+      </c>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E16" s="22" t="n">
+        <v>6236.25</v>
+      </c>
+      <c r="F16" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G16" s="21" t="n"/>
+      <c r="I16" s="20" t="inlineStr">
+        <is>
+          <t>6826210</t>
+        </is>
+      </c>
+      <c r="J16" s="22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C17" s="21" t="n">
+        <v>1200393</v>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E17" s="22" t="n">
+        <v>29236.55</v>
+      </c>
+      <c r="F17" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G17" s="21" t="n"/>
+      <c r="I17" s="20" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="J17" s="22" t="n">
+        <v>545.78</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="n">
+        <v>1200393</v>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E18" s="22" t="n">
+        <v>5853.45</v>
+      </c>
+      <c r="F18" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G18" s="21" t="n"/>
+      <c r="I18" s="20" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="J18" s="22" t="n">
+        <v>338.38</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="n">
+        <v>1040211</v>
+      </c>
+      <c r="D19" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E19" s="22" t="n">
+        <v>17918.3</v>
+      </c>
+      <c r="F19" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G19" s="21" t="n"/>
+      <c r="I19" s="20" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="J19" s="22" t="n">
+        <v>184.21</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="n">
+        <v>21</v>
+      </c>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C20" s="21" t="n">
+        <v>1170144</v>
+      </c>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E20" s="22" t="n">
+        <v>338.38</v>
+      </c>
+      <c r="F20" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G20" s="21" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="n">
+        <v>22</v>
+      </c>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C21" s="21" t="n">
+        <v>1040109</v>
+      </c>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E21" s="22" t="n">
+        <v>282.67</v>
+      </c>
+      <c r="F21" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G21" s="21" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="20" t="n">
+        <v>23</v>
+      </c>
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C22" s="21" t="n">
+        <v>1040109</v>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="n">
+        <v>19637.26</v>
+      </c>
+      <c r="F22" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G22" s="21" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C23" s="21" t="n">
+        <v>1170144</v>
+      </c>
+      <c r="D23" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E23" s="22" t="n">
+        <v>184.21</v>
+      </c>
+      <c r="F23" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G23" s="21" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="n">
+        <v>26</v>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C24" s="21" t="n">
+        <v>1040375</v>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E24" s="22" t="n">
+        <v>417.36</v>
+      </c>
+      <c r="F24" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G24" s="21" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="n">
+        <v>27</v>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C25" s="21" t="n">
+        <v>1040375</v>
+      </c>
+      <c r="D25" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E25" s="22" t="n">
+        <v>128.42</v>
+      </c>
+      <c r="F25" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G25" s="21" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="n">
+        <v>33</v>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>Pagamento</t>
+        </is>
+      </c>
+      <c r="C26" s="21" t="n">
+        <v>1040258</v>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>27/jul/26</t>
+        </is>
+      </c>
+      <c r="E26" s="22" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="F26" s="21" t="inlineStr">
+        <is>
+          <t>Não reconciliado</t>
+        </is>
+      </c>
+      <c r="G26" s="21" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="I8:J8"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>